<commit_message>
Add baseline CNN notebook with PyTorch, update results
</commit_message>
<xml_diff>
--- a/results/result.xlsx
+++ b/results/result.xlsx
@@ -1,61 +1,88 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HUSSAIN\OneDrive\Desktop\cnn-architecture-comparison-cifar10\results\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF14972C-016A-4799-AEBB-D4B9F519C380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>Test Accuracy (%)</t>
+  </si>
+  <si>
+    <t>Trainable Parameters</t>
+  </si>
+  <si>
+    <t>Training Time (s)</t>
+  </si>
+  <si>
+    <t>Baseline CNN</t>
+  </si>
+  <si>
+    <t>84,586</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
+      <sz val="11"/>
       <name val="Arial"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="FFD6E4F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,106 +96,51 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -456,123 +428,103 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Test Accuracy (%)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Trainable Parameters</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Training Time (s)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Baseline CNN</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>84,586</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>75.46</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr"/>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="3" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
+    <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0.68259999999999998</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2">
+        <v>646.52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Resnet18 and VGG11 notebooks with results
</commit_message>
<xml_diff>
--- a/results/result.xlsx
+++ b/results/result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HUSSAIN\OneDrive\Desktop\cnn-architecture-comparison-cifar10\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF14972C-016A-4799-AEBB-D4B9F519C380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B57DFB9-7286-4CA9-AFFB-CB1E7B776DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Architecture</t>
   </si>
@@ -37,14 +37,29 @@
     <t>Baseline CNN</t>
   </si>
   <si>
-    <t>84,586</t>
+    <t>ResNet18</t>
+  </si>
+  <si>
+    <t>VGG11</t>
+  </si>
+  <si>
+    <t>DenseNet121</t>
+  </si>
+  <si>
+    <t>306.58 seconds(5.10966667 minutes)</t>
+  </si>
+  <si>
+    <t>290.77 seconds(4.84616667 minutes)</t>
+  </si>
+  <si>
+    <t>254.05 seconds(4.234 minutes)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,8 +77,15 @@
       <sz val="11"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -83,6 +105,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -125,6 +153,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -434,8 +474,8 @@
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" customWidth="1"/>
+    <col min="4" max="4" width="37.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -457,29 +497,47 @@
         <v>4</v>
       </c>
       <c r="B2" s="4">
-        <v>0.68259999999999998</v>
-      </c>
-      <c r="C2" s="2" t="s">
+        <v>0.74160000000000004</v>
+      </c>
+      <c r="C2" s="8">
+        <v>620810</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
-        <v>646.52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="B3" s="6">
+        <v>0.67230000000000001</v>
+      </c>
+      <c r="C3" s="7">
+        <v>11181642</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.60089999999999999</v>
+      </c>
+      <c r="C4" s="8">
+        <v>9359882</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -528,5 +586,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add CIFAR-100 experiments for CNN, ResNet18 and VGG11
</commit_message>
<xml_diff>
--- a/results/result.xlsx
+++ b/results/result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HUSSAIN\OneDrive\Desktop\cnn-architecture-comparison-cifar10\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B57DFB9-7286-4CA9-AFFB-CB1E7B776DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9480B15C-939F-4F02-847F-CC954069409C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,11 +20,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Architecture</t>
   </si>
   <si>
+    <t>Dataset</t>
+  </si>
+  <si>
     <t>Test Accuracy (%)</t>
   </si>
   <si>
@@ -37,13 +40,55 @@
     <t>Baseline CNN</t>
   </si>
   <si>
+    <t>CIFAR-10</t>
+  </si>
+  <si>
+    <t>74.16%</t>
+  </si>
+  <si>
+    <t>620,810</t>
+  </si>
+  <si>
     <t>ResNet18</t>
   </si>
   <si>
+    <t>67.23%</t>
+  </si>
+  <si>
+    <t>11,181,642</t>
+  </si>
+  <si>
     <t>VGG11</t>
   </si>
   <si>
-    <t>DenseNet121</t>
+    <t>60.09%</t>
+  </si>
+  <si>
+    <t>9,359,882</t>
+  </si>
+  <si>
+    <t>CIFAR-100</t>
+  </si>
+  <si>
+    <t>39.05%</t>
+  </si>
+  <si>
+    <t>31.25%</t>
+  </si>
+  <si>
+    <t>11,227,812</t>
+  </si>
+  <si>
+    <t>10.45%</t>
+  </si>
+  <si>
+    <t>278.19 seconds(4.6365 minutes)</t>
+  </si>
+  <si>
+    <t>257.80 seconds(4.29666667 minutes)</t>
+  </si>
+  <si>
+    <t>254.05 seconds(4.234 minutes)</t>
   </si>
   <si>
     <t>306.58 seconds(5.10966667 minutes)</t>
@@ -52,14 +97,14 @@
     <t>290.77 seconds(4.84616667 minutes)</t>
   </si>
   <si>
-    <t>254.05 seconds(4.234 minutes)</t>
+    <t>321.36305.75 seconds(5.09583333 minutes)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -77,15 +122,8 @@
       <sz val="11"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -105,12 +143,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -141,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -152,19 +184,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -469,16 +489,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="24.88671875" customWidth="1"/>
-    <col min="4" max="4" width="37.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="47.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,101 +512,113 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4">
-        <v>0.74160000000000004</v>
-      </c>
-      <c r="C2" s="8">
-        <v>620810</v>
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="4" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6">
-        <v>0.67230000000000001</v>
-      </c>
-      <c r="C3" s="7">
-        <v>11181642</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="B5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="E5" s="3" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="4" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="4">
-        <v>0.60089999999999999</v>
-      </c>
-      <c r="C4" s="8">
-        <v>9359882</v>
-      </c>
-      <c r="D4" s="2" t="s">
+    <row r="6" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-    </row>
-    <row r="6" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-    </row>
-    <row r="10" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+    <row r="7" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="4">
+        <v>9383012</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>